<commit_message>
etsy: planejador de mudanca (tarefas datadas a partir do dia, caixas numeradas por comodo, orcamentos de transportadoras, custos, quem avisar do novo endereco); festa: total do dinheiro soma todos os custos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DYz1Azd3FHBSgFnLhXfMUY
</commit_message>
<xml_diff>
--- a/etsy/party/Party-Planner.xlsx
+++ b/etsy/party/Party-Planner.xlsx
@@ -1768,15 +1768,15 @@
         </is>
       </c>
       <c r="C33" s="27">
-        <f>SUM(C22:C32)</f>
+        <f>SUM(Budget!$M$6:$M$55)+SUM('Food and drinks'!$K$8:$K$47)</f>
         <v/>
       </c>
       <c r="D33" s="27">
-        <f>SUM(D22:D32)</f>
+        <f>SUM(Budget!$G$6:$G$55)+SUMIFS('Food and drinks'!$K$8:$K$47,'Food and drinks'!$L$8:$L$47,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="E33" s="27">
-        <f>SUM(E22:E32)</f>
+        <f>SUM(Budget!$H$6:$H$55)+SUM('Food and drinks'!$K$8:$K$47)-SUMIFS('Food and drinks'!$K$8:$K$47,'Food and drinks'!$L$8:$L$47,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="F33" s="1" t="n"/>

</xml_diff>